<commit_message>
Harden public-repo ignores and placeholder samples
Ignore local editor settings, switch credential examples to explicit placeholders, and replace long synthetic fixture reference numbers with clearly fake IDs so publication scrub scans stay quiet.
</commit_message>
<xml_diff>
--- a/tests/fixtures/amex_activity_sanitized.xlsx
+++ b/tests/fixtures/amex_activity_sanitized.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>320260070187470819</t>
+          <t>REF-20260106-01</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>320260050078449011</t>
+          <t>REF-20260105-01</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>320260040078923435</t>
+          <t>REF-20260104-01</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">

</xml_diff>